<commit_message>
plantillas: propuesta comercial automática dentro del diagnóstico
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019RbM9k9qVMfLYsqfpAZa9N
</commit_message>
<xml_diff>
--- a/plantillas/diagnostico-financiero-pyme.xlsx
+++ b/plantillas/diagnostico-financiero-pyme.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Diagnostico" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Datos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Parametros" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Propuesta" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Datos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Parametros" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Diagnostico'!$A$1:$F$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Propuesta'!$A$1:$F$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28,7 +30,7 @@
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +79,30 @@
       <i val="1"/>
       <sz val="8"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+    </font>
+    <font>
+      <color rgb="00808080"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -122,18 +148,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -141,6 +174,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -151,6 +185,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -165,11 +214,14 @@
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <font>
         <b val="1"/>
@@ -223,6 +275,9 @@
           <fgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="0.0%"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -658,7 +713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -684,475 +739,541 @@
     </row>
     <row r="3">
       <c r="A3">
-        <f>"Periodo: "&amp;Datos!B6&amp;"   ·   Régimen: "&amp;Datos!B5&amp;"   ·   Fecha: "&amp;TEXT(Datos!B7,"dd/mm/yyyy")</f>
+        <f>"Periodo: "&amp;Datos!B6&amp;"   ·   Régimen: "&amp;Datos!B5</f>
+        <v/>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Fecha:</t>
+        </is>
+      </c>
+      <c r="F3" s="6">
+        <f>Datos!B7</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>CIFRAS CLAVE</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Ventas</t>
         </is>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <f>Datos!B11</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Utilidad bruta</t>
         </is>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="9">
         <f>Datos!B11-Datos!B12</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Utilidad operacional (EBIT)</t>
         </is>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="9">
         <f>Datos!B11-Datos!B12-Datos!B13-Datos!B14</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Utilidad neta</t>
         </is>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="9">
         <f>Datos!B11-Datos!B12-Datos!B13-Datos!B14-Datos!B15+Datos!B16-Datos!B17</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Activo total</t>
         </is>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="9">
         <f>SUM(Datos!B20:B24)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Pasivo total</t>
         </is>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="9">
         <f>SUM(Datos!B25:B29)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Patrimonio</t>
         </is>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="9">
         <f>B10-B11</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Verde si</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Rojo si</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>Semáforo</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>Acción recomendada</t>
         </is>
       </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Orden</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="6">
+      <c r="A15" s="8">
         <f>Parametros!A2</f>
         <v/>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="12">
         <f>IFERROR(B7/Datos!B11,"N/D")</f>
         <v/>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="12">
         <f>Parametros!C2</f>
         <v/>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="12">
         <f>Parametros!D2</f>
         <v/>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="13">
         <f>IF(ISNUMBER(B15),IF(Parametros!B2=1,IF(B15&gt;=C15,"Verde",IF(B15&lt;D15,"Rojo","Amarillo")),IF(B15&lt;=C15,"Verde",IF(B15&gt;D15,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="14">
         <f>IF(E15="Rojo",Parametros!E2,IF(E15="Amarillo",Parametros!F2,IF(E15="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G15" s="15">
+        <f>IF(E15="Rojo",COUNTIF(E$15:E15,"Rojo"),IF(E15="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E15,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="6">
+      <c r="A16" s="8">
         <f>Parametros!A3</f>
         <v/>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="12">
         <f>IFERROR(B8/Datos!B11,"N/D")</f>
         <v/>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="12">
         <f>Parametros!C3</f>
         <v/>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="12">
         <f>Parametros!D3</f>
         <v/>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="13">
         <f>IF(ISNUMBER(B16),IF(Parametros!B3=1,IF(B16&gt;=C16,"Verde",IF(B16&lt;D16,"Rojo","Amarillo")),IF(B16&lt;=C16,"Verde",IF(B16&gt;D16,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="14">
         <f>IF(E16="Rojo",Parametros!E3,IF(E16="Amarillo",Parametros!F3,IF(E16="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G16" s="15">
+        <f>IF(E16="Rojo",COUNTIF(E$15:E16,"Rojo"),IF(E16="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E16,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="6">
+      <c r="A17" s="8">
         <f>Parametros!A4</f>
         <v/>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="12">
         <f>IFERROR(B9/Datos!B11,"N/D")</f>
         <v/>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="12">
         <f>Parametros!C4</f>
         <v/>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="12">
         <f>Parametros!D4</f>
         <v/>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="13">
         <f>IF(ISNUMBER(B17),IF(Parametros!B4=1,IF(B17&gt;=C17,"Verde",IF(B17&lt;D17,"Rojo","Amarillo")),IF(B17&lt;=C17,"Verde",IF(B17&gt;D17,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="14">
         <f>IF(E17="Rojo",Parametros!E4,IF(E17="Amarillo",Parametros!F4,IF(E17="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G17" s="15">
+        <f>IF(E17="Rojo",COUNTIF(E$15:E17,"Rojo"),IF(E17="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E17,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="6">
+      <c r="A18" s="8">
         <f>Parametros!A5</f>
         <v/>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="16">
         <f>IFERROR(SUM(Datos!B20:B23)/SUM(Datos!B25:B28),"N/D")</f>
         <v/>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="16">
         <f>Parametros!C5</f>
         <v/>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="16">
         <f>Parametros!D5</f>
         <v/>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="13">
         <f>IF(ISNUMBER(B18),IF(Parametros!B5=1,IF(B18&gt;=C18,"Verde",IF(B18&lt;D18,"Rojo","Amarillo")),IF(B18&lt;=C18,"Verde",IF(B18&gt;D18,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="14">
         <f>IF(E18="Rojo",Parametros!E5,IF(E18="Amarillo",Parametros!F5,IF(E18="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G18" s="15">
+        <f>IF(E18="Rojo",COUNTIF(E$15:E18,"Rojo"),IF(E18="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E18,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6">
+      <c r="A19" s="8">
         <f>Parametros!A6</f>
         <v/>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="16">
         <f>IFERROR((SUM(Datos!B20:B23)-Datos!B22)/SUM(Datos!B25:B28),"N/D")</f>
         <v/>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="16">
         <f>Parametros!C6</f>
         <v/>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="16">
         <f>Parametros!D6</f>
         <v/>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="13">
         <f>IF(ISNUMBER(B19),IF(Parametros!B6=1,IF(B19&gt;=C19,"Verde",IF(B19&lt;D19,"Rojo","Amarillo")),IF(B19&lt;=C19,"Verde",IF(B19&gt;D19,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F19" s="11">
+      <c r="F19" s="14">
         <f>IF(E19="Rojo",Parametros!E6,IF(E19="Amarillo",Parametros!F6,IF(E19="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G19" s="15">
+        <f>IF(E19="Rojo",COUNTIF(E$15:E19,"Rojo"),IF(E19="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E19,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="6">
+      <c r="A20" s="8">
         <f>Parametros!A7</f>
         <v/>
       </c>
-      <c r="B20" s="13">
+      <c r="B20" s="17">
         <f>IFERROR(Datos!B21/Datos!B11*365,"N/D")</f>
         <v/>
       </c>
-      <c r="C20" s="13">
+      <c r="C20" s="17">
         <f>Parametros!C7</f>
         <v/>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="17">
         <f>Parametros!D7</f>
         <v/>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="13">
         <f>IF(ISNUMBER(B20),IF(Parametros!B7=1,IF(B20&gt;=C20,"Verde",IF(B20&lt;D20,"Rojo","Amarillo")),IF(B20&lt;=C20,"Verde",IF(B20&gt;D20,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F20" s="11">
+      <c r="F20" s="14">
         <f>IF(E20="Rojo",Parametros!E7,IF(E20="Amarillo",Parametros!F7,IF(E20="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G20" s="15">
+        <f>IF(E20="Rojo",COUNTIF(E$15:E20,"Rojo"),IF(E20="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E20,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="6">
+      <c r="A21" s="8">
         <f>Parametros!A8</f>
         <v/>
       </c>
-      <c r="B21" s="13">
+      <c r="B21" s="17">
         <f>IFERROR(Datos!B22/Datos!B12*365,"N/D")</f>
         <v/>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="17">
         <f>Parametros!C8</f>
         <v/>
       </c>
-      <c r="D21" s="13">
+      <c r="D21" s="17">
         <f>Parametros!D8</f>
         <v/>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="13">
         <f>IF(ISNUMBER(B21),IF(Parametros!B8=1,IF(B21&gt;=C21,"Verde",IF(B21&lt;D21,"Rojo","Amarillo")),IF(B21&lt;=C21,"Verde",IF(B21&gt;D21,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="14">
         <f>IF(E21="Rojo",Parametros!E8,IF(E21="Amarillo",Parametros!F8,IF(E21="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G21" s="15">
+        <f>IF(E21="Rojo",COUNTIF(E$15:E21,"Rojo"),IF(E21="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E21,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="6">
+      <c r="A22" s="8">
         <f>Parametros!A9</f>
         <v/>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="17">
         <f>IFERROR(Datos!B25/Datos!B12*365,"N/D")</f>
         <v/>
       </c>
-      <c r="C22" s="13">
+      <c r="C22" s="17">
         <f>Parametros!C9</f>
         <v/>
       </c>
-      <c r="D22" s="13">
+      <c r="D22" s="17">
         <f>Parametros!D9</f>
         <v/>
       </c>
-      <c r="E22" s="10">
+      <c r="E22" s="13">
         <f>IF(ISNUMBER(B22),IF(Parametros!B9=1,IF(B22&gt;=C22,"Verde",IF(B22&lt;D22,"Rojo","Amarillo")),IF(B22&lt;=C22,"Verde",IF(B22&gt;D22,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="14">
         <f>IF(E22="Rojo",Parametros!E9,IF(E22="Amarillo",Parametros!F9,IF(E22="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G22" s="15">
+        <f>IF(E22="Rojo",COUNTIF(E$15:E22,"Rojo"),IF(E22="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E22,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="6">
+      <c r="A23" s="8">
         <f>Parametros!A10</f>
         <v/>
       </c>
-      <c r="B23" s="13">
+      <c r="B23" s="17">
         <f>IFERROR(B20+B21-B22,"N/D")</f>
         <v/>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="17">
         <f>Parametros!C10</f>
         <v/>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="17">
         <f>Parametros!D10</f>
         <v/>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="13">
         <f>IF(ISNUMBER(B23),IF(Parametros!B10=1,IF(B23&gt;=C23,"Verde",IF(B23&lt;D23,"Rojo","Amarillo")),IF(B23&lt;=C23,"Verde",IF(B23&gt;D23,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="14">
         <f>IF(E23="Rojo",Parametros!E10,IF(E23="Amarillo",Parametros!F10,IF(E23="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G23" s="15">
+        <f>IF(E23="Rojo",COUNTIF(E$15:E23,"Rojo"),IF(E23="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E23,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="6">
+      <c r="A24" s="8">
         <f>Parametros!A11</f>
         <v/>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="12">
         <f>IFERROR(B11/B10,"N/D")</f>
         <v/>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="12">
         <f>Parametros!C11</f>
         <v/>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="12">
         <f>Parametros!D11</f>
         <v/>
       </c>
-      <c r="E24" s="10">
+      <c r="E24" s="13">
         <f>IF(ISNUMBER(B24),IF(Parametros!B11=1,IF(B24&gt;=C24,"Verde",IF(B24&lt;D24,"Rojo","Amarillo")),IF(B24&lt;=C24,"Verde",IF(B24&gt;D24,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F24" s="11">
+      <c r="F24" s="14">
         <f>IF(E24="Rojo",Parametros!E11,IF(E24="Amarillo",Parametros!F11,IF(E24="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G24" s="15">
+        <f>IF(E24="Rojo",COUNTIF(E$15:E24,"Rojo"),IF(E24="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E24,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="6">
+      <c r="A25" s="8">
         <f>Parametros!A12</f>
         <v/>
       </c>
-      <c r="B25" s="14">
+      <c r="B25" s="18">
         <f>IFERROR(B8/Datos!B15,"N/D")</f>
         <v/>
       </c>
-      <c r="C25" s="14">
+      <c r="C25" s="18">
         <f>Parametros!C12</f>
         <v/>
       </c>
-      <c r="D25" s="14">
+      <c r="D25" s="18">
         <f>Parametros!D12</f>
         <v/>
       </c>
-      <c r="E25" s="10">
+      <c r="E25" s="13">
         <f>IF(ISNUMBER(B25),IF(Parametros!B12=1,IF(B25&gt;=C25,"Verde",IF(B25&lt;D25,"Rojo","Amarillo")),IF(B25&lt;=C25,"Verde",IF(B25&gt;D25,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="14">
         <f>IF(E25="Rojo",Parametros!E12,IF(E25="Amarillo",Parametros!F12,IF(E25="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G25" s="15">
+        <f>IF(E25="Rojo",COUNTIF(E$15:E25,"Rojo"),IF(E25="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E25,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="6">
+      <c r="A26" s="8">
         <f>Parametros!A13</f>
         <v/>
       </c>
-      <c r="B26" s="14">
+      <c r="B26" s="18">
         <f>IFERROR(Datos!B20/Datos!B31,"N/D")</f>
         <v/>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="18">
         <f>Parametros!C13</f>
         <v/>
       </c>
-      <c r="D26" s="14">
+      <c r="D26" s="18">
         <f>Parametros!D13</f>
         <v/>
       </c>
-      <c r="E26" s="10">
+      <c r="E26" s="13">
         <f>IF(ISNUMBER(B26),IF(Parametros!B13=1,IF(B26&gt;=C26,"Verde",IF(B26&lt;D26,"Rojo","Amarillo")),IF(B26&lt;=C26,"Verde",IF(B26&gt;D26,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F26" s="11">
+      <c r="F26" s="14">
         <f>IF(E26="Rojo",Parametros!E13,IF(E26="Amarillo",Parametros!F13,IF(E26="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G26" s="15">
+        <f>IF(E26="Rojo",COUNTIF(E$15:E26,"Rojo"),IF(E26="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E26,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="6">
+      <c r="A27" s="8">
         <f>Parametros!A14</f>
         <v/>
       </c>
-      <c r="B27" s="15">
+      <c r="B27" s="19">
         <f>IFERROR(COUNTIF(Datos!B34:B43,"Sí")/(COUNTIF(Datos!B34:B43,"Sí")+COUNTIF(Datos!B34:B43,"No")),"N/D")</f>
         <v/>
       </c>
-      <c r="C27" s="15">
+      <c r="C27" s="19">
         <f>Parametros!C14</f>
         <v/>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="19">
         <f>Parametros!D14</f>
         <v/>
       </c>
-      <c r="E27" s="10">
+      <c r="E27" s="13">
         <f>IF(ISNUMBER(B27),IF(Parametros!B14=1,IF(B27&gt;=C27,"Verde",IF(B27&lt;D27,"Rojo","Amarillo")),IF(B27&lt;=C27,"Verde",IF(B27&gt;D27,"Rojo","Amarillo"))),"N/D")</f>
         <v/>
       </c>
-      <c r="F27" s="11">
+      <c r="F27" s="14">
         <f>IF(E27="Rojo",Parametros!E14,IF(E27="Amarillo",Parametros!F14,IF(E27="Verde","Mantener.","Falta información.")))</f>
         <v/>
       </c>
+      <c r="G27" s="15">
+        <f>IF(E27="Rojo",COUNTIF(E$15:E27,"Rojo"),IF(E27="Amarillo",COUNTIF($E$15:$E$27,"Rojo")+COUNTIF(E$15:E27,"Amarillo"),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>PUNTAJE DE SALUD FINANCIERA</t>
         </is>
       </c>
-      <c r="B29" s="16">
+      <c r="B29" s="20">
         <f>IFERROR((COUNTIF(E15:E27,"Verde")*2+COUNTIF(E15:E27,"Amarillo"))/((COUNTIF(E15:E27,"Verde")+COUNTIF(E15:E27,"Amarillo")+COUNTIF(E15:E27,"Rojo"))*2),0)</f>
         <v/>
       </c>
-      <c r="C29" s="17">
+      <c r="C29" s="21">
         <f>IF(B29&gt;=0.75,"SALUDABLE",IF(B29&gt;=0.5,"EN ALERTA","CRÍTICO"))</f>
         <v/>
       </c>
@@ -1169,21 +1290,21 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>PRÓXIMO PASO RECOMENDADO</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="18">
+      <c r="A33" s="22">
         <f>IF(COUNTIF(E15:E27,"Rojo")&gt;=3,"Acompañamiento financiero mensual: hay "&amp;COUNTIF(E15:E27,"Rojo")&amp;" indicadores críticos que requieren seguimiento continuo.",IF(COUNTIF(E15:E27,"Rojo")&gt;=1,"Plan de acción de 90 días sobre los indicadores en rojo, con revisión mensual.","Seguimiento trimestral y planeación tributaria para proteger la rentabilidad."))</f>
         <v/>
       </c>
     </row>
     <row r="34"/>
     <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>Diagnóstico basado en la información suministrada por el cliente, sin auditar. Rangos de referencia generales.</t>
         </is>
@@ -1194,7 +1315,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A33:F34"/>
   </mergeCells>
   <conditionalFormatting sqref="E15:E27">
@@ -1229,6 +1350,531 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>PROPUESTA DE SERVICIOS CONTABLES Y FINANCIEROS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>"Para: "&amp;Datos!B2&amp;"   ·   NIT: "&amp;Datos!B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Fecha:</t>
+        </is>
+      </c>
+      <c r="B3" s="6">
+        <f>Datos!B7</f>
+        <v/>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Válida hasta:</t>
+        </is>
+      </c>
+      <c r="D3" s="6">
+        <f>Datos!B7+Parametros!B33</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>Parametros!B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>1. SITUACIÓN ENCONTRADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Salud financiera</t>
+        </is>
+      </c>
+      <c r="B6" s="26">
+        <f>Diagnostico!B29</f>
+        <v/>
+      </c>
+      <c r="C6" s="7">
+        <f>Diagnostico!C29</f>
+        <v/>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rojo / amarillo / verde</t>
+        </is>
+      </c>
+      <c r="F6">
+        <f>Diagnostico!B30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Hallazgo prioritario</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Qué haremos</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="8">
+        <f>IFERROR(INDEX(Diagnostico!$A$15:$A$27,MATCH(1,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B8" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$B$15:$B$27,MATCH(1,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$C$15:$C$27,MATCH(1,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="13">
+        <f>IFERROR(INDEX(Diagnostico!$E$15:$E$27,MATCH(1,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="14">
+        <f>IFERROR(INDEX(Diagnostico!$F$15:$F$27,MATCH(1,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="15">
+        <f>IFERROR(INDEX(Parametros!$G$2:$G$14,MATCH(1,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="8">
+        <f>IFERROR(INDEX(Diagnostico!$A$15:$A$27,MATCH(2,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B9" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$B$15:$B$27,MATCH(2,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$C$15:$C$27,MATCH(2,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D9" s="13">
+        <f>IFERROR(INDEX(Diagnostico!$E$15:$E$27,MATCH(2,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="14">
+        <f>IFERROR(INDEX(Diagnostico!$F$15:$F$27,MATCH(2,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="15">
+        <f>IFERROR(INDEX(Parametros!$G$2:$G$14,MATCH(2,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="8">
+        <f>IFERROR(INDEX(Diagnostico!$A$15:$A$27,MATCH(3,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B10" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$B$15:$B$27,MATCH(3,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C10" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$C$15:$C$27,MATCH(3,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="13">
+        <f>IFERROR(INDEX(Diagnostico!$E$15:$E$27,MATCH(3,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="14">
+        <f>IFERROR(INDEX(Diagnostico!$F$15:$F$27,MATCH(3,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="15">
+        <f>IFERROR(INDEX(Parametros!$G$2:$G$14,MATCH(3,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="8">
+        <f>IFERROR(INDEX(Diagnostico!$A$15:$A$27,MATCH(4,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B11" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$B$15:$B$27,MATCH(4,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$C$15:$C$27,MATCH(4,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D11" s="13">
+        <f>IFERROR(INDEX(Diagnostico!$E$15:$E$27,MATCH(4,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="14">
+        <f>IFERROR(INDEX(Diagnostico!$F$15:$F$27,MATCH(4,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="15">
+        <f>IFERROR(INDEX(Parametros!$G$2:$G$14,MATCH(4,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="8">
+        <f>IFERROR(INDEX(Diagnostico!$A$15:$A$27,MATCH(5,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B12" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$B$15:$B$27,MATCH(5,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="18">
+        <f>IFERROR(INDEX(Diagnostico!$C$15:$C$27,MATCH(5,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="13">
+        <f>IFERROR(INDEX(Diagnostico!$E$15:$E$27,MATCH(5,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="14">
+        <f>IFERROR(INDEX(Diagnostico!$F$15:$F$27,MATCH(5,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="15">
+        <f>IFERROR(INDEX(Parametros!$G$2:$G$14,MATCH(5,Diagnostico!$G$15:$G$27,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>2. CAJA QUE SE PUEDE LIBERAR (estimación)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cartera por encima de la meta</t>
+        </is>
+      </c>
+      <c r="B15" s="27">
+        <f>IF(ISNUMBER(Diagnostico!B20),MAX(0,Diagnostico!B20-Diagnostico!C20)*Datos!B11/365,0)</f>
+        <v/>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>Dinero inmovilizado en cartera e inventario por encima de los días meta. Llevar esos días a la meta libera esa caja sin endeudarse. Es una estimación basada en las cifras del periodo; el resultado real depende de la ejecución.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Inventario por encima de la meta</t>
+        </is>
+      </c>
+      <c r="B16" s="27">
+        <f>IF(ISNUMBER(Diagnostico!B21),MAX(0,Diagnostico!B21-Diagnostico!C21)*Datos!B12/365,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Total caja potencial</t>
+        </is>
+      </c>
+      <c r="B17" s="29">
+        <f>B15+B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>3. PLAN RECOMENDADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Plan sugerido por el diagnóstico</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>IF(COUNTIF(Diagnostico!$E$15:$E$27,"Rojo")&gt;=3,"CFO fraccional",IF(COUNTIF(Diagnostico!$E$15:$E$27,"Rojo")&gt;=1,"Crecimiento","Empresa"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Plan propuesto</t>
+        </is>
+      </c>
+      <c r="B21" s="30">
+        <f>IF(Datos!B9&lt;&gt;"",Datos!B9,B20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Incluye</t>
+        </is>
+      </c>
+      <c r="B22" s="31">
+        <f>IFERROR(VLOOKUP(B21,Parametros!$A$21:$C$24,3,FALSE),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>4. CÓMO TRABAJAREMOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Semana 1</t>
+        </is>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Recepción de información y accesos al software contable; plan de normalización de los hallazgos en rojo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Semanas 2–4</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>Puesta al día contable y tributaria; primeras acciones sobre cartera, inventario y caja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Cada mes</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="inlineStr">
+        <is>
+          <t>Cierre contable, declaraciones a tiempo e informe con indicadores y semáforo (este mismo formato).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Mes 3</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="inlineStr">
+        <is>
+          <t>Revisión de resultados frente a este diagnóstico: ¿cuánta caja se liberó y qué indicadores mejoraron?</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>5. INVERSIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Valor mensual</t>
+        </is>
+      </c>
+      <c r="B32" s="29">
+        <f>IFERROR(VLOOKUP(B21,Parametros!$A$21:$B$24,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="C32" s="32">
+        <f>IF(AND(ISNUMBER(B32),B17&gt;0),B32*12/B17,"")</f>
+        <v/>
+      </c>
+      <c r="D32" s="33" t="inlineStr">
+        <is>
+          <t>del valor anual frente a la caja potencial a liberar</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="B33" s="31">
+        <f>Parametros!B34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>6. PRÓXIMO PASO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>Para iniciar: (1) aceptar esta propuesta respondiendo este mensaje o firmando abajo, (2) realizar el primer pago y (3) enviar la información contable y los accesos. Iniciamos en los 3 días hábiles siguientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>_____________________________</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>_____________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <f>Parametros!B28</f>
+        <v/>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aceptado por: </t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <f>"Contador Público · "&amp;Parametros!B29</f>
+        <v/>
+      </c>
+      <c r="D42">
+        <f>Datos!B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="34">
+        <f>Parametros!B30&amp;" · "&amp;Parametros!B31</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A36:F37"/>
+    <mergeCell ref="B22:F23"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="C15:F17"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B8:C12">
+    <cfRule type="expression" priority="1" dxfId="6">
+      <formula>$G8="pct"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D8:D12">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="2">
+      <formula>"Rojo"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"Amarillo"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C43"/>
@@ -1240,7 +1886,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="35" t="inlineStr">
         <is>
           <t>DATOS DEL CLIENTE</t>
         </is>
@@ -1252,7 +1898,7 @@
           <t>Empresa</t>
         </is>
       </c>
-      <c r="B2" s="21" t="inlineStr">
+      <c r="B2" s="36" t="inlineStr">
         <is>
           <t>Comercializadora Ejemplo SAS</t>
         </is>
@@ -1264,7 +1910,7 @@
           <t>NIT</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>901000000-1</t>
         </is>
@@ -1276,7 +1922,7 @@
           <t>Sector</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="36" t="inlineStr">
         <is>
           <t>Comercio</t>
         </is>
@@ -1288,7 +1934,7 @@
           <t>Régimen</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="36" t="inlineStr">
         <is>
           <t>Ordinario</t>
         </is>
@@ -1300,7 +1946,7 @@
           <t>Periodo analizado</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="36" t="inlineStr">
         <is>
           <t>Ene–Dic 2025</t>
         </is>
@@ -1312,7 +1958,7 @@
           <t>Fecha del diagnóstico</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="37" t="n">
         <v>46311</v>
       </c>
     </row>
@@ -1322,459 +1968,470 @@
           <t>Elaborado por</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="36" t="inlineStr">
         <is>
           <t>Contador Público TP ____</t>
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Plan elegido (opcional; vacío = recomendado)</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n"/>
+    </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>ESTADO DE RESULTADOS (periodo)</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Valor COP</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Ventas netas</t>
         </is>
       </c>
-      <c r="B11" s="23" t="n">
+      <c r="B11" s="38" t="n">
         <v>1200000000</v>
       </c>
-      <c r="C11" s="6" t="inlineStr"/>
+      <c r="C11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Costo de ventas</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="38" t="n">
         <v>840000000</v>
       </c>
-      <c r="C12" s="6" t="inlineStr"/>
+      <c r="C12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Gastos de administración</t>
         </is>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="38" t="n">
         <v>150000000</v>
       </c>
-      <c r="C13" s="6" t="inlineStr"/>
+      <c r="C13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Gastos de ventas</t>
         </is>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="38" t="n">
         <v>95000000</v>
       </c>
-      <c r="C14" s="6" t="inlineStr"/>
+      <c r="C14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Gastos financieros (intereses)</t>
         </is>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="38" t="n">
         <v>38000000</v>
       </c>
-      <c r="C15" s="6" t="inlineStr"/>
+      <c r="C15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Otros ingresos (gastos) netos</t>
         </is>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Positivo = ingreso</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Impuesto de renta</t>
         </is>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="38" t="n">
         <v>25000000</v>
       </c>
-      <c r="C17" s="6" t="inlineStr"/>
+      <c r="C17" s="8" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>BALANCE (fecha de corte)</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Valor COP</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Efectivo y equivalentes</t>
         </is>
       </c>
-      <c r="B20" s="23" t="n">
+      <c r="B20" s="38" t="n">
         <v>35000000</v>
       </c>
-      <c r="C20" s="6" t="inlineStr"/>
+      <c r="C20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Cuentas por cobrar clientes</t>
         </is>
       </c>
-      <c r="B21" s="23" t="n">
+      <c r="B21" s="38" t="n">
         <v>260000000</v>
       </c>
-      <c r="C21" s="6" t="inlineStr"/>
+      <c r="C21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Inventarios</t>
         </is>
       </c>
-      <c r="B22" s="23" t="n">
+      <c r="B22" s="38" t="n">
         <v>180000000</v>
       </c>
-      <c r="C22" s="6" t="inlineStr"/>
+      <c r="C22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Otros activos corrientes</t>
         </is>
       </c>
-      <c r="B23" s="23" t="n">
+      <c r="B23" s="38" t="n">
         <v>20000000</v>
       </c>
-      <c r="C23" s="6" t="inlineStr"/>
+      <c r="C23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Activos no corrientes (propiedad, planta, otros)</t>
         </is>
       </c>
-      <c r="B24" s="23" t="n">
+      <c r="B24" s="38" t="n">
         <v>210000000</v>
       </c>
-      <c r="C24" s="6" t="inlineStr"/>
+      <c r="C24" s="8" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Proveedores</t>
         </is>
       </c>
-      <c r="B25" s="23" t="n">
+      <c r="B25" s="38" t="n">
         <v>95000000</v>
       </c>
-      <c r="C25" s="6" t="inlineStr"/>
+      <c r="C25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Obligaciones financieras corto plazo</t>
         </is>
       </c>
-      <c r="B26" s="23" t="n">
+      <c r="B26" s="38" t="n">
         <v>140000000</v>
       </c>
-      <c r="C26" s="6" t="inlineStr"/>
+      <c r="C26" s="8" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Impuestos por pagar</t>
         </is>
       </c>
-      <c r="B27" s="23" t="n">
+      <c r="B27" s="38" t="n">
         <v>30000000</v>
       </c>
-      <c r="C27" s="6" t="inlineStr"/>
+      <c r="C27" s="8" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>Otros pasivos corrientes</t>
         </is>
       </c>
-      <c r="B28" s="23" t="n">
+      <c r="B28" s="38" t="n">
         <v>25000000</v>
       </c>
-      <c r="C28" s="6" t="inlineStr"/>
+      <c r="C28" s="8" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Pasivos no corrientes</t>
         </is>
       </c>
-      <c r="B29" s="23" t="n">
+      <c r="B29" s="38" t="n">
         <v>120000000</v>
       </c>
-      <c r="C29" s="6" t="inlineStr"/>
+      <c r="C29" s="8" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Gasto fijo mensual promedio (nómina, arriendo, servicios…)</t>
         </is>
       </c>
-      <c r="B31" s="23" t="n">
+      <c r="B31" s="38" t="n">
         <v>22000000</v>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Para calcular los meses de caja disponibles</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>CHEQUEO TRIBUTARIO</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Sí / No / N/A</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>Riesgo si es 'No'</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>RUT actualizado (responsabilidades y actividad)</t>
         </is>
       </c>
-      <c r="B34" s="24" t="inlineStr">
+      <c r="B34" s="39" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>Sanciones / responsabilidades mal asignadas</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>Facturación electrónica habilitada y emitiendo</t>
         </is>
       </c>
-      <c r="B35" s="24" t="inlineStr">
+      <c r="B35" s="39" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Sanción por no facturar; rechazo de costos del cliente</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Nómina electrónica transmitida mensualmente</t>
         </is>
       </c>
-      <c r="B36" s="24" t="inlineStr">
+      <c r="B36" s="39" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>Costos de nómina no deducibles</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>Documento soporte en compras a no obligados</t>
         </is>
       </c>
-      <c r="B37" s="24" t="inlineStr">
+      <c r="B37" s="39" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Costos y gastos no deducibles</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>Retenciones en la fuente declaradas y pagadas a tiempo</t>
         </is>
       </c>
-      <c r="B38" s="24" t="inlineStr">
+      <c r="B38" s="39" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>Ineficacia de la declaración + intereses</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>IVA / impuesto al consumo declarado a tiempo</t>
         </is>
       </c>
-      <c r="B39" s="24" t="inlineStr">
+      <c r="B39" s="39" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>Sanción por extemporaneidad e intereses</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Renta del último año presentada</t>
         </is>
       </c>
-      <c r="B40" s="24" t="inlineStr">
+      <c r="B40" s="39" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>Omisión / emplazamiento DIAN</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>Información exógena reportada</t>
         </is>
       </c>
-      <c r="B41" s="24" t="inlineStr">
+      <c r="B41" s="39" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>Sanción por no enviar información</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>ICA / industria y comercio al día</t>
         </is>
       </c>
-      <c r="B42" s="24" t="inlineStr">
+      <c r="B42" s="39" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>Sanciones municipales</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>Contabilidad al día (cierre mensual ≤ 30 días)</t>
         </is>
       </c>
-      <c r="B43" s="24" t="inlineStr">
+      <c r="B43" s="39" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>Decisiones con información atrasada</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"SIMPLE,Ordinario,Persona natural,No responsable de IVA"</formula1>
     </dataValidation>
     <dataValidation sqref="B34 B35 B36 B37 B38 B39 B40 B41 B42 B43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No,N/A"</formula1>
     </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=Parametros!$A$21:$A$24</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1786,383 +2443,634 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>Verde si</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>Rojo si</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>Acción si ROJO</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>Acción si AMARILLO</t>
         </is>
       </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Margen bruto</t>
         </is>
       </c>
-      <c r="B2" s="25" t="n">
+      <c r="B2" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="26" t="n">
+      <c r="C2" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="D2" s="26" t="n">
+      <c r="D2" s="41" t="n">
         <v>0.2</v>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>Revisar precios, descuentos y costo de compra; el margen no cubre la operación.</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr">
         <is>
           <t>Negociar con proveedores y revisar la mezcla de productos.</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Margen operacional</t>
         </is>
       </c>
-      <c r="B3" s="25" t="n">
+      <c r="B3" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="26" t="n">
+      <c r="C3" s="41" t="n">
         <v>0.1</v>
       </c>
-      <c r="D3" s="26" t="n">
+      <c r="D3" s="41" t="n">
         <v>0.03</v>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>Los gastos consumen el margen: recortar gastos fijos y revisar la estructura.</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>Controlar los gastos de administración y ventas mes a mes.</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Margen neto</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
+      <c r="B4" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="26" t="n">
+      <c r="C4" s="41" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="D4" s="41" t="n">
         <v>0.02</v>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>La rentabilidad final es crítica: revisar la carga financiera y tributaria.</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>Planeación tributaria y reducción del costo financiero.</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Razón corriente</t>
         </is>
       </c>
-      <c r="B5" s="25" t="n">
+      <c r="B5" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="42" t="n">
         <v>1.5</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Riesgo de iliquidez: los pasivos de corto plazo superan los activos corrientes.</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>Mejorar el capital de trabajo: cobrar más rápido y reestructurar la deuda de corto plazo.</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Prueba ácida</t>
         </is>
       </c>
-      <c r="B6" s="25" t="n">
+      <c r="B6" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="42" t="n">
         <v>0.7</v>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Sin inventario no alcanza a cubrir las deudas de corto plazo.</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>Reducir el inventario inmovilizado.</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Días de cartera</t>
         </is>
       </c>
-      <c r="B7" s="25" t="n">
+      <c r="B7" s="40" t="n">
         <v>-1</v>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="43" t="n">
         <v>45</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="D7" s="43" t="n">
         <v>90</v>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Los clientes pagan muy tarde: política de crédito, cobro y descuentos por pronto pago.</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>Seguimiento semanal de la cartera por edades.</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Días de inventario</t>
         </is>
       </c>
-      <c r="B8" s="25" t="n">
+      <c r="B8" s="40" t="n">
         <v>-1</v>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="43" t="n">
         <v>60</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="43" t="n">
         <v>120</v>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Exceso de inventario: liquidar las referencias de baja rotación.</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>Ajustar las compras a la rotación real.</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Días de proveedores</t>
         </is>
       </c>
-      <c r="B9" s="25" t="n">
+      <c r="B9" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="43" t="n">
         <v>30</v>
       </c>
-      <c r="D9" s="28" t="n">
+      <c r="D9" s="43" t="n">
         <v>15</v>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Pagas demasiado rápido: negociar plazos con los proveedores.</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>Buscar más plazo con los proveedores clave.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Ciclo de caja (días)</t>
         </is>
       </c>
-      <c r="B10" s="25" t="n">
+      <c r="B10" s="40" t="n">
         <v>-1</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="43" t="n">
         <v>45</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="43" t="n">
         <v>90</v>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>El negocio financia a los clientes durante demasiado tiempo: actuar sobre cartera, inventario y proveedores.</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>Monitorear el ciclo de caja mensualmente.</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Endeudamiento</t>
         </is>
       </c>
-      <c r="B11" s="25" t="n">
+      <c r="B11" s="40" t="n">
         <v>-1</v>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="41" t="n">
         <v>0.5</v>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D11" s="41" t="n">
         <v>0.7</v>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>Deuda alta: frenar el endeudamiento nuevo y reestructurar.</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>Vigilar el nivel de deuda antes de financiar crecimiento.</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Cobertura de intereses</t>
         </is>
       </c>
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="29" t="n">
+      <c r="C12" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="44" t="n">
         <v>1.5</v>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>La utilidad operativa apenas cubre los intereses: refinanciar.</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="14" t="inlineStr">
         <is>
           <t>Buscar tasas más bajas o prepagar la deuda cara.</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Meses de caja</t>
         </is>
       </c>
-      <c r="B13" s="25" t="n">
+      <c r="B13" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="29" t="n">
+      <c r="C13" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Menos de 1 mes de caja: plan de tesorería urgente (flujo a 13 semanas).</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Construir una reserva de al menos 3 meses de gastos fijos.</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Cumplimiento tributario</t>
         </is>
       </c>
-      <c r="B14" s="25" t="n">
+      <c r="B14" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="30" t="n">
+      <c r="C14" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="30" t="n">
+      <c r="D14" s="45" t="n">
         <v>0.8</v>
       </c>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Riesgo alto de sanciones DIAN: normalizar las obligaciones pendientes de inmediato.</t>
         </is>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Corregir los puntos pendientes del chequeo tributario.</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="46" t="inlineStr">
         <is>
           <t>Dirección: 1 = más alto es mejor · -1 = más bajo es mejor. Los rangos son referencias generales; ajústalos por sector.</t>
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Precio mensual</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Incluye</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr"/>
+      <c r="F20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Básico</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="n">
+        <v>450000</v>
+      </c>
+      <c r="C21" s="47" t="inlineStr">
+        <is>
+          <t>Contabilidad mensual, declaraciones tributarias y facturación electrónica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="B22" s="38" t="n">
+        <v>750000</v>
+      </c>
+      <c r="C22" s="47" t="inlineStr">
+        <is>
+          <t>Básico + nómina electrónica, retenciones, información exógena e informe mensual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Crecimiento</t>
+        </is>
+      </c>
+      <c r="B23" s="38" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="C23" s="47" t="inlineStr">
+        <is>
+          <t>Empresa + flujo de caja, presupuesto, indicadores y reunión mensual de resultados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>CFO fraccional</t>
+        </is>
+      </c>
+      <c r="B24" s="38" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="C24" s="47" t="inlineStr">
+        <is>
+          <t>Crecimiento + flujo de caja a 13 semanas, gestión de cartera e inventario, análisis de precios y márgenes, y acompañamiento en decisiones financieras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Datos del contador</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr"/>
+      <c r="C27" s="10" t="inlineStr"/>
+      <c r="D27" s="10" t="inlineStr"/>
+      <c r="E27" s="10" t="inlineStr"/>
+      <c r="F27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="inlineStr">
+        <is>
+          <t>[Tu nombre]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Tarjeta profesional</t>
+        </is>
+      </c>
+      <c r="B29" s="36" t="inlineStr">
+        <is>
+          <t>TP ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Teléfono / WhatsApp</t>
+        </is>
+      </c>
+      <c r="B30" s="36" t="inlineStr">
+        <is>
+          <t>[300 000 0000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
+      <c r="B31" s="36" t="inlineStr">
+        <is>
+          <t>[correo@dominio.com]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Ciudad</t>
+        </is>
+      </c>
+      <c r="B32" s="36" t="inlineStr">
+        <is>
+          <t>Montería</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Validez de la propuesta (días)</t>
+        </is>
+      </c>
+      <c r="B33" s="36" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Condiciones de pago</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="inlineStr">
+        <is>
+          <t>Pago anticipado del día 1 al 5 de cada mes. Atraso mayor de 15 días suspende el servicio. Valores antes de IVA, si aplica.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C24:F24"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>